<commit_message>
Close Plan v5.0.0 and Account Plan v1.1.0: new design
Close plan: one-page Summary tab (score, bucket bars, top risks, next actions,
key people, deal story) driven by formulas into the other tabs; workbook restyled
in the Aircover palette; Action Plan filters. Scoring unchanged.
Account plan: At a glance first page and restyled document.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/close-plan/assets/Close_Plan_TEMPLATE.xlsx
+++ b/close-plan/assets/Close_Plan_TEMPLATE.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health Score" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Plan" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder Map" sheetId="4" state="visible" r:id="rId4"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,35 +31,102 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FF2CB5AD"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF7A8CA0"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2CB5AD"/>
+      <sz val="28"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF7A8CA0"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF7A8CA0"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF2CB5AD"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFD94F4F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF3D4F6F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2CB5AD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF3D4F6F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF1E1E1E"/>
+      <color rgb="FF2CB5AD"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="FF666666"/>
+      <i val="1"/>
+      <color rgb="FF7A8CA0"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -70,31 +137,35 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFF6C37"/>
-      <sz val="10"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="9"/>
+      <color rgb="FF1E7B55"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFF6C37"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <color rgb="FF8A6100"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFB23B3B"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -103,36 +174,41 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FF2CB5AD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF6C37"/>
+        <fgColor rgb="FFF7F9FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E1E1E"/>
+        <fgColor rgb="FFE8ECF0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor rgb="FFE3F5EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFFDF3D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE4E4"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -140,65 +216,163 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FF2CB5AD"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -563,125 +737,610 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="B1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Close Plan for:</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>AE:</t>
-        </is>
-      </c>
+    <row r="1" ht="4" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>CRM:</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>SE:</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Close Date:</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Partner:</t>
-        </is>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CLOSE PLAN</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>CLOSE READINESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="B3" s="4" t="n"/>
+      <c r="H3" s="5">
+        <f>'Health Score'!B3</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Net Incremental ARR</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Deal in Forecast:</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>DEAL SYNOPSIS &amp; OVERVIEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>share of the 26 checklist items</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>AMOUNT</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>CLOSE DATE</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>STAGE</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>PARTNER</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>READINESS BY BUCKET</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Stakeholder Alignment</t>
+        </is>
+      </c>
+      <c r="D10" s="14">
+        <f>REPT("█",ROUND('Health Score'!C7*36,0))</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
+        <f>'Health Score'!C7</f>
+        <v/>
+      </c>
+      <c r="I10" s="16">
+        <f>IF(H10=MIN($H$10:$H$14),"Weakest","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Technical Validation</t>
+        </is>
+      </c>
+      <c r="D11" s="14">
+        <f>REPT("█",ROUND('Health Score'!C15*36,0))</f>
+        <v/>
+      </c>
+      <c r="H11" s="15">
+        <f>'Health Score'!C15</f>
+        <v/>
+      </c>
+      <c r="I11" s="16">
+        <f>IF(H11=MIN($H$10:$H$14),"Weakest","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D12" s="14">
+        <f>REPT("█",ROUND('Health Score'!C21*36,0))</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>'Health Score'!C21</f>
+        <v/>
+      </c>
+      <c r="I12" s="16">
+        <f>IF(H12=MIN($H$10:$H$14),"Weakest","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="D13" s="14">
+        <f>REPT("█",ROUND('Health Score'!C29*36,0))</f>
+        <v/>
+      </c>
+      <c r="H13" s="15">
+        <f>'Health Score'!C29</f>
+        <v/>
+      </c>
+      <c r="I13" s="16">
+        <f>IF(H13=MIN($H$10:$H$14),"Weakest","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Timeline &amp; Risk</t>
+        </is>
+      </c>
+      <c r="D14" s="14">
+        <f>REPT("█",ROUND('Health Score'!C34*36,0))</f>
+        <v/>
+      </c>
+      <c r="H14" s="15">
+        <f>'Health Score'!C34</f>
+        <v/>
+      </c>
+      <c r="I14" s="16">
+        <f>IF(H14=MIN($H$10:$H$14),"Weakest","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>TOP RISKS</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="17" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="17" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="17" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>NEXT ACTIONS</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="12" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>ACTION</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>OWNER</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="20" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="21" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="20" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="21" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="21" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="21" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="21" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>KEY PEOPLE</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>ENGAGEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="22">
+        <f>'Stakeholder Map'!A18</f>
+        <v/>
+      </c>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="23">
+        <f>'Stakeholder Map'!B18</f>
+        <v/>
+      </c>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="24">
+        <f>'Stakeholder Map'!C18</f>
+        <v/>
+      </c>
+      <c r="I31" s="12" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="22">
+        <f>'Stakeholder Map'!A19</f>
+        <v/>
+      </c>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="23">
+        <f>'Stakeholder Map'!B19</f>
+        <v/>
+      </c>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="24">
+        <f>'Stakeholder Map'!C19</f>
+        <v/>
+      </c>
+      <c r="I32" s="12" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="22">
+        <f>'Stakeholder Map'!A20</f>
+        <v/>
+      </c>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="23">
+        <f>'Stakeholder Map'!B20</f>
+        <v/>
+      </c>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="24">
+        <f>'Stakeholder Map'!C20</f>
+        <v/>
+      </c>
+      <c r="I33" s="12" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="22">
+        <f>'Stakeholder Map'!A21</f>
+        <v/>
+      </c>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="23">
+        <f>'Stakeholder Map'!B21</f>
+        <v/>
+      </c>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="24">
+        <f>'Stakeholder Map'!C21</f>
+        <v/>
+      </c>
+      <c r="I34" s="12" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="22">
+        <f>'Stakeholder Map'!A22</f>
+        <v/>
+      </c>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="23">
+        <f>'Stakeholder Map'!B22</f>
+        <v/>
+      </c>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="24">
+        <f>'Stakeholder Map'!C22</f>
+        <v/>
+      </c>
+      <c r="I35" s="12" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="22">
+        <f>'Stakeholder Map'!A23</f>
+        <v/>
+      </c>
+      <c r="C36" s="12" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="23">
+        <f>'Stakeholder Map'!B23</f>
+        <v/>
+      </c>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="24">
+        <f>'Stakeholder Map'!C23</f>
+        <v/>
+      </c>
+      <c r="I36" s="12" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>DEAL STORY</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>Who are the primary business units using the product?</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="69.75" customHeight="1">
-      <c r="A8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="B40" s="17" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>How are they using the product today?</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="69.75" customHeight="1">
-      <c r="A10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="17" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>What is the primary use case vs. what is the secondary use case? (use case = what problem are we solving)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="69.75" customHeight="1">
-      <c r="A12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="17" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>What is the product's impact to the customer's business? (cite specific metrics)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="69.75" customHeight="1">
-      <c r="A14" s="4" t="n"/>
-    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="B46" s="17" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="B48" s="26">
+        <f>IF('Health Score'!A44="","",'Health Score'!A44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
+  <mergeCells count="57">
+    <mergeCell ref="B48:I49"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="G7:I7"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -689,313 +1348,339 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>HEALTH SCORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Overall Close Plan Score</t>
-        </is>
-      </c>
-      <c r="B3" s="7">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Health Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B3" s="29">
         <f>AVERAGE(C7,C15,C21,C29,C34)</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="41" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Key: every item scored "No", "In Progress" or "Needs Input" generates a recommended action in the Action Plan tab. "Yes" items are validated and get no bullet there, which keeps this tab scannable. Each item is worth an equal share of its bucket: Yes = 100%, In Progress = 50%, No and Needs Input = 0%. Overall = the five bucket scores weighted equally.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Every item scored "No", "In Progress" or "Needs Input" generates a recommended action on the Action Plan tab. Each item is worth an equal share of its bucket: Yes = 100%, In Progress = 50%, No and Needs Input = 0%. Overall = the five bucket scores weighted equally. Change a status from the dropdown and every score, including the Summary, recalculates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>STAKEHOLDER ALIGNMENT</t>
         </is>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="32">
         <f>(COUNTIF(A8:A13,"Yes")+0.5*COUNTIF(A8:A13,"In Progress"))/COUNTA($B$8:$B$13)</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="33" t="n"/>
+      <c r="B8" s="34" t="inlineStr">
         <is>
           <t>Champion identified and confirmed (has influence + is actively selling internally)</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="C8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="33" t="n"/>
+      <c r="B9" s="34" t="inlineStr">
         <is>
           <t>Economic buyer identified and engaged directly (not just through champion)</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C9" s="12" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="33" t="n"/>
+      <c r="B10" s="34" t="inlineStr">
         <is>
           <t>All stakeholders/influencers mapped (security, legal, procurement, end users, IT)</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="C10" s="12" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="33" t="n"/>
+      <c r="B11" s="34" t="inlineStr">
         <is>
           <t>Decision criteria documented and agreed by buyer</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="C11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="33" t="n"/>
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>Decision process and approval chain confirmed (who signs, in what order)</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="C12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="33" t="n"/>
+      <c r="B13" s="34" t="inlineStr">
         <is>
           <t>Compelling event / reason to act by target date is explicit</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="C13" s="12" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>TECHNICAL VALIDATION</t>
         </is>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="32">
         <f>(COUNTIF(A16:A19,"Yes")+0.5*COUNTIF(A16:A19,"In Progress"))/COUNTA($B$16:$B$19)</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="33" t="n"/>
+      <c r="B16" s="34" t="inlineStr">
         <is>
           <t>Technical win confirmed (POC/trial success criteria met and documented)</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="C16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="33" t="n"/>
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>Security review status known (in progress / passed / not started)</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="C17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="33" t="n"/>
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>Integration requirements scoped and no blockers open</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="C18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="33" t="n"/>
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>Any outstanding product gaps or feature requests flagged to product team</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="C19" s="12" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>COMMERCIAL</t>
         </is>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="32">
         <f>(COUNTIF(A22:A27,"Yes")+0.5*COUNTIF(A22:A27,"In Progress"))/COUNTA($B$22:$B$27)</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="33" t="n"/>
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>Budget confirmed to exist and be allocated for this fiscal period</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="C22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="33" t="n"/>
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Pricing/packaging aligned with buyer's expectations</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="C23" s="12" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="33" t="n"/>
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>Quote/order form sent and reviewed by buyer</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="C24" s="12" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="33" t="n"/>
+      <c r="B25" s="34" t="inlineStr">
         <is>
           <t>Procurement process started (vendor onboarding, security questionnaires, etc.)</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="11" t="n"/>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="C25" s="12" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="33" t="n"/>
+      <c r="B26" s="34" t="inlineStr">
         <is>
           <t>Legal/MSA redlines identified early, not first surfaced at the finish line</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="C26" s="12" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="33" t="n"/>
+      <c r="B27" s="34" t="inlineStr">
         <is>
           <t>Have we established enough value w/ key stakeholders to mitigate potential for discounting?</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="C27" s="12" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="31" t="inlineStr">
         <is>
           <t>COMPETITION</t>
         </is>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="32">
         <f>(COUNTIF(A30:A32,"Yes")+0.5*COUNTIF(A30:A32,"In Progress"))/COUNTA($B$30:$B$32)</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="4" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="34" t="inlineStr">
         <is>
           <t>Competitive landscape known (incumbent, alternatives being evaluated)</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="C30" s="12" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="33" t="n"/>
+      <c r="B31" s="34" t="inlineStr">
         <is>
           <t>Differentiation validated with champion, they can repeat it internally</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="C31" s="12" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="33" t="n"/>
+      <c r="B32" s="34" t="inlineStr">
         <is>
           <t>No unaddressed objections tied to a competitor's pitch</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="C32" s="12" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t>TIMELINE &amp; RISK</t>
         </is>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="32">
         <f>(COUNTIF(A35:A41,"Yes")+0.5*COUNTIF(A35:A41,"In Progress"))/COUNTA($B$35:$B$41)</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="4" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="33" t="n"/>
+      <c r="B35" s="34" t="inlineStr">
         <is>
           <t>Mutual close plan shared with buyer, with dates both sides agreed to</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="11" t="n"/>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="C35" s="12" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="33" t="n"/>
+      <c r="B36" s="34" t="inlineStr">
         <is>
           <t>Next step scheduled with a specific date (not "follow up next week")</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="C36" s="12" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="33" t="n"/>
+      <c r="B37" s="34" t="inlineStr">
         <is>
           <t>Key risk(s) to close named explicitly, e.g. budget freeze, exec turnover, competing priority</t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="11" t="n"/>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="C37" s="12" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="33" t="n"/>
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>Backup plan if primary champion goes dark or leaves</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="C38" s="12" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="33" t="n"/>
+      <c r="B39" s="34" t="inlineStr">
         <is>
           <t>Do we have a clear migration or onboarding plan?</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="11" t="n"/>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="C39" s="12" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="33" t="n"/>
+      <c r="B40" s="34" t="inlineStr">
         <is>
           <t>Do we have an onboarding owner identified?</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="11" t="n"/>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="C40" s="12" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="33" t="n"/>
+      <c r="B41" s="34" t="inlineStr">
         <is>
           <t>Forecast category matches actual deal signals (don't call it Commit if 3+ boxes above are unchecked)</t>
         </is>
       </c>
+      <c r="C41" s="12" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="A43" s="35" t="inlineStr">
         <is>
           <t>COVERAGE AND EVIDENCE LIMITS</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14.5" customHeight="1">
-      <c r="A44" s="13" t="n"/>
+      <c r="A44" s="36" t="n"/>
     </row>
     <row r="45" ht="14.5" customHeight="1"/>
     <row r="46" ht="14.5" customHeight="1"/>
@@ -1016,7 +1701,8 @@
       <formula1>"Yes,No,In Progress,Needs Input"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1024,68 +1710,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>ACTION PLAN: one row per Health Score item that is not a Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Action Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="37" t="inlineStr">
+        <is>
+          <t>One row per Health Score item that is not a Yes. Filter by owner or status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="31" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="31" t="inlineStr">
         <is>
           <t>Gap (from Health Score)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="31" t="inlineStr">
         <is>
           <t>Recommended Action</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="31" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="31" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="31" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1093,7 +1784,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1107,244 +1798,268 @@
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>STAKEHOLDER MAP: heat map of persona engagement</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Buying Committee Heat Map: seniority x function</t>
-        </is>
-      </c>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Stakeholder Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t>BUYING COMMITTEE: seniority x function</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="n"/>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="12" t="n"/>
+      <c r="E3" s="12" t="n"/>
+      <c r="F3" s="12" t="n"/>
+      <c r="G3" s="12" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>C-Suite</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
-    </row>
-    <row r="7" ht="27.75" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="B5" s="40" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Seniority</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Business / LOB</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Technical / Engineering</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>Enablement / Ops</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="F7" s="41" t="inlineStr">
         <is>
           <t>IT / Platform</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="G7" s="41" t="inlineStr">
         <is>
           <t>Procurement / Legal</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>VP</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
+      <c r="B8" s="43" t="n"/>
+      <c r="C8" s="43" t="n"/>
+      <c r="D8" s="43" t="n"/>
+      <c r="E8" s="43" t="n"/>
+      <c r="F8" s="43" t="n"/>
+      <c r="G8" s="43" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
+      <c r="B9" s="43" t="n"/>
+      <c r="C9" s="43" t="n"/>
+      <c r="D9" s="43" t="n"/>
+      <c r="E9" s="43" t="n"/>
+      <c r="F9" s="43" t="n"/>
+      <c r="G9" s="43" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="18" t="n"/>
-      <c r="G10" s="18" t="n"/>
+      <c r="B10" s="43" t="n"/>
+      <c r="C10" s="43" t="n"/>
+      <c r="D10" s="43" t="n"/>
+      <c r="E10" s="43" t="n"/>
+      <c r="F10" s="43" t="n"/>
+      <c r="G10" s="43" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Individual Contributor</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
+      <c r="B11" s="43" t="n"/>
+      <c r="C11" s="43" t="n"/>
+      <c r="D11" s="43" t="n"/>
+      <c r="E11" s="43" t="n"/>
+      <c r="F11" s="43" t="n"/>
+      <c r="G11" s="43" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="42" t="inlineStr">
         <is>
           <t>Seniority not stated</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Key:</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B12" s="43" t="n"/>
+      <c r="C12" s="43" t="n"/>
+      <c r="D12" s="43" t="n"/>
+      <c r="E12" s="43" t="n"/>
+      <c r="F12" s="43" t="n"/>
+      <c r="G12" s="43" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="inlineStr">
         <is>
           <t>Engaged</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="46" t="inlineStr">
         <is>
           <t>Emerging / not direct</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="47" t="inlineStr">
         <is>
           <t>Not yet mapped</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25.5" customHeight="1"/>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Key Persona Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>KEY PERSONAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>Engagement</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="31" t="inlineStr">
         <is>
           <t>Notes / Gap</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="39.75" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="49" t="inlineStr">
         <is>
           <t>Economic Buyer</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="39.75" customHeight="1">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="49" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="39.75" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="33" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="49" t="inlineStr">
         <is>
           <t>Executive Sponsor</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="39.75" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="49" t="inlineStr">
         <is>
           <t>Influencer 1 - Security / Legal</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="39.75" customHeight="1">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="20" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="49" t="inlineStr">
         <is>
           <t>Influencer 2 - Procurement</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="39.75" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
+      <c r="B22" s="20" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="20" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="49" t="inlineStr">
         <is>
           <t>Influencer 3 - End Users / IT</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="4" t="n"/>
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="20" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="50" t="inlineStr">
         <is>
           <t>Open question: Do we have a text relationship with any of these contacts?</t>
         </is>
@@ -1370,6 +2085,7 @@
       <formula1>"Engaged,Emerging,Not yet mapped"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add README screenshots; solid bucket bars and cleaner table headers
Close plan Summary bars are now Excel data bars written solid by the engine
(block characters showed seams). Account plan table headers no longer show a
white seam between cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/close-plan/assets/Close_Plan_TEMPLATE.xlsx
+++ b/close-plan/assets/Close_Plan_TEMPLATE.xlsx
@@ -19,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="24">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode=";;;"/>
+  </numFmts>
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,11 +70,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FF1B2A4A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="FF2CB5AD"/>
       <sz val="10"/>
     </font>
     <font>
@@ -208,7 +205,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -224,6 +221,14 @@
     <border>
       <bottom style="thin">
         <color rgb="FFE2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thick">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFFFFFFF"/>
       </bottom>
     </border>
     <border>
@@ -244,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -275,35 +280,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -312,63 +316,63 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -866,14 +870,17 @@
         </is>
       </c>
       <c r="D10" s="14">
-        <f>REPT("█",ROUND('Health Score'!C7*36,0))</f>
-        <v/>
-      </c>
-      <c r="H10" s="15">
         <f>'Health Score'!C7</f>
         <v/>
       </c>
-      <c r="I10" s="16">
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="16">
+        <f>'Health Score'!C7</f>
+        <v/>
+      </c>
+      <c r="I10" s="17">
         <f>IF(H10=MIN($H$10:$H$14),"Weakest","")</f>
         <v/>
       </c>
@@ -885,14 +892,17 @@
         </is>
       </c>
       <c r="D11" s="14">
-        <f>REPT("█",ROUND('Health Score'!C15*36,0))</f>
-        <v/>
-      </c>
-      <c r="H11" s="15">
         <f>'Health Score'!C15</f>
         <v/>
       </c>
-      <c r="I11" s="16">
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="16">
+        <f>'Health Score'!C15</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
         <f>IF(H11=MIN($H$10:$H$14),"Weakest","")</f>
         <v/>
       </c>
@@ -904,14 +914,17 @@
         </is>
       </c>
       <c r="D12" s="14">
-        <f>REPT("█",ROUND('Health Score'!C21*36,0))</f>
-        <v/>
-      </c>
-      <c r="H12" s="15">
         <f>'Health Score'!C21</f>
         <v/>
       </c>
-      <c r="I12" s="16">
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="16">
+        <f>'Health Score'!C21</f>
+        <v/>
+      </c>
+      <c r="I12" s="17">
         <f>IF(H12=MIN($H$10:$H$14),"Weakest","")</f>
         <v/>
       </c>
@@ -923,14 +936,17 @@
         </is>
       </c>
       <c r="D13" s="14">
-        <f>REPT("█",ROUND('Health Score'!C29*36,0))</f>
-        <v/>
-      </c>
-      <c r="H13" s="15">
         <f>'Health Score'!C29</f>
         <v/>
       </c>
-      <c r="I13" s="16">
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="16">
+        <f>'Health Score'!C29</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
         <f>IF(H13=MIN($H$10:$H$14),"Weakest","")</f>
         <v/>
       </c>
@@ -942,14 +958,17 @@
         </is>
       </c>
       <c r="D14" s="14">
-        <f>REPT("█",ROUND('Health Score'!C34*36,0))</f>
-        <v/>
-      </c>
-      <c r="H14" s="15">
         <f>'Health Score'!C34</f>
         <v/>
       </c>
-      <c r="I14" s="16">
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="16">
+        <f>'Health Score'!C34</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
         <f>IF(H14=MIN($H$10:$H$14),"Weakest","")</f>
         <v/>
       </c>
@@ -969,13 +988,13 @@
       <c r="I16" s="12" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="17" t="n"/>
+      <c r="B17" s="18" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="17" t="n"/>
+      <c r="B18" s="18" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="17" t="n"/>
+      <c r="B19" s="18" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="11" t="inlineStr">
@@ -992,86 +1011,86 @@
       <c r="I21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>ACTION</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>OWNER</t>
         </is>
       </c>
-      <c r="I22" s="18" t="inlineStr">
+      <c r="I22" s="19" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="19" t="n">
+      <c r="B23" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="20" t="n"/>
+      <c r="C23" s="21" t="n"/>
       <c r="D23" s="12" t="n"/>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="12" t="n"/>
-      <c r="G23" s="20" t="n"/>
+      <c r="G23" s="21" t="n"/>
       <c r="H23" s="12" t="n"/>
-      <c r="I23" s="21" t="n"/>
+      <c r="I23" s="22" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="B24" s="19" t="n">
+      <c r="B24" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="20" t="n"/>
+      <c r="C24" s="21" t="n"/>
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="12" t="n"/>
       <c r="F24" s="12" t="n"/>
-      <c r="G24" s="20" t="n"/>
+      <c r="G24" s="21" t="n"/>
       <c r="H24" s="12" t="n"/>
-      <c r="I24" s="21" t="n"/>
+      <c r="I24" s="22" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="19" t="n">
+      <c r="B25" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="20" t="n"/>
+      <c r="C25" s="21" t="n"/>
       <c r="D25" s="12" t="n"/>
       <c r="E25" s="12" t="n"/>
       <c r="F25" s="12" t="n"/>
-      <c r="G25" s="20" t="n"/>
+      <c r="G25" s="21" t="n"/>
       <c r="H25" s="12" t="n"/>
-      <c r="I25" s="21" t="n"/>
+      <c r="I25" s="22" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="20" t="n"/>
+      <c r="C26" s="21" t="n"/>
       <c r="D26" s="12" t="n"/>
       <c r="E26" s="12" t="n"/>
       <c r="F26" s="12" t="n"/>
-      <c r="G26" s="20" t="n"/>
+      <c r="G26" s="21" t="n"/>
       <c r="H26" s="12" t="n"/>
-      <c r="I26" s="21" t="n"/>
+      <c r="I26" s="22" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="20" t="n"/>
+      <c r="C27" s="21" t="n"/>
       <c r="D27" s="12" t="n"/>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="12" t="n"/>
-      <c r="G27" s="20" t="n"/>
+      <c r="G27" s="21" t="n"/>
       <c r="H27" s="12" t="n"/>
-      <c r="I27" s="21" t="n"/>
+      <c r="I27" s="22" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
@@ -1088,131 +1107,131 @@
       <c r="I29" s="12" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>ROLE</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="H30" s="18" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>ENGAGEMENT</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="22">
+      <c r="B31" s="23">
         <f>'Stakeholder Map'!A18</f>
         <v/>
       </c>
       <c r="C31" s="12" t="n"/>
       <c r="D31" s="12" t="n"/>
-      <c r="E31" s="23">
+      <c r="E31" s="24">
         <f>'Stakeholder Map'!B18</f>
         <v/>
       </c>
       <c r="F31" s="12" t="n"/>
       <c r="G31" s="12" t="n"/>
-      <c r="H31" s="24">
+      <c r="H31" s="25">
         <f>'Stakeholder Map'!C18</f>
         <v/>
       </c>
       <c r="I31" s="12" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="22">
+      <c r="B32" s="23">
         <f>'Stakeholder Map'!A19</f>
         <v/>
       </c>
       <c r="C32" s="12" t="n"/>
       <c r="D32" s="12" t="n"/>
-      <c r="E32" s="23">
+      <c r="E32" s="24">
         <f>'Stakeholder Map'!B19</f>
         <v/>
       </c>
       <c r="F32" s="12" t="n"/>
       <c r="G32" s="12" t="n"/>
-      <c r="H32" s="24">
+      <c r="H32" s="25">
         <f>'Stakeholder Map'!C19</f>
         <v/>
       </c>
       <c r="I32" s="12" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="22">
+      <c r="B33" s="23">
         <f>'Stakeholder Map'!A20</f>
         <v/>
       </c>
       <c r="C33" s="12" t="n"/>
       <c r="D33" s="12" t="n"/>
-      <c r="E33" s="23">
+      <c r="E33" s="24">
         <f>'Stakeholder Map'!B20</f>
         <v/>
       </c>
       <c r="F33" s="12" t="n"/>
       <c r="G33" s="12" t="n"/>
-      <c r="H33" s="24">
+      <c r="H33" s="25">
         <f>'Stakeholder Map'!C20</f>
         <v/>
       </c>
       <c r="I33" s="12" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="B34" s="22">
+      <c r="B34" s="23">
         <f>'Stakeholder Map'!A21</f>
         <v/>
       </c>
       <c r="C34" s="12" t="n"/>
       <c r="D34" s="12" t="n"/>
-      <c r="E34" s="23">
+      <c r="E34" s="24">
         <f>'Stakeholder Map'!B21</f>
         <v/>
       </c>
       <c r="F34" s="12" t="n"/>
       <c r="G34" s="12" t="n"/>
-      <c r="H34" s="24">
+      <c r="H34" s="25">
         <f>'Stakeholder Map'!C21</f>
         <v/>
       </c>
       <c r="I34" s="12" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="22">
+      <c r="B35" s="23">
         <f>'Stakeholder Map'!A22</f>
         <v/>
       </c>
       <c r="C35" s="12" t="n"/>
       <c r="D35" s="12" t="n"/>
-      <c r="E35" s="23">
+      <c r="E35" s="24">
         <f>'Stakeholder Map'!B22</f>
         <v/>
       </c>
       <c r="F35" s="12" t="n"/>
       <c r="G35" s="12" t="n"/>
-      <c r="H35" s="24">
+      <c r="H35" s="25">
         <f>'Stakeholder Map'!C22</f>
         <v/>
       </c>
       <c r="I35" s="12" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="22">
+      <c r="B36" s="23">
         <f>'Stakeholder Map'!A23</f>
         <v/>
       </c>
       <c r="C36" s="12" t="n"/>
       <c r="D36" s="12" t="n"/>
-      <c r="E36" s="23">
+      <c r="E36" s="24">
         <f>'Stakeholder Map'!B23</f>
         <v/>
       </c>
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="12" t="n"/>
-      <c r="H36" s="24">
+      <c r="H36" s="25">
         <f>'Stakeholder Map'!C23</f>
         <v/>
       </c>
@@ -1233,47 +1252,47 @@
       <c r="I38" s="12" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="25" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>Who are the primary business units using the product?</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="B40" s="17" t="n"/>
+      <c r="B40" s="18" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>How are they using the product today?</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="B42" s="17" t="n"/>
+      <c r="B42" s="18" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="B43" s="25" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>What is the primary use case vs. what is the secondary use case? (use case = what problem are we solving)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="17" t="n"/>
+      <c r="B44" s="18" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="25" t="inlineStr">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>What is the product's impact to the customer's business? (cite specific metrics)</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="B46" s="17" t="n"/>
+      <c r="B46" s="18" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="B48" s="26">
+      <c r="B48" s="27">
         <f>IF('Health Score'!A44="","",'Health Score'!A44)</f>
         <v/>
       </c>
@@ -1339,6 +1358,15 @@
     <mergeCell ref="B41:I41"/>
     <mergeCell ref="G7:I7"/>
   </mergeCells>
+  <conditionalFormatting sqref="D10:D14">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="0">
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="002CB5AD"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1359,44 +1387,44 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Health Score</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>Overall</t>
         </is>
       </c>
-      <c r="B3" s="29">
+      <c r="B3" s="30">
         <f>AVERAGE(C7,C15,C21,C29,C34)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Every item scored "No", "In Progress" or "Needs Input" generates a recommended action on the Action Plan tab. Each item is worth an equal share of its bucket: Yes = 100%, In Progress = 50%, No and Needs Input = 0%. Overall = the five bucket scores weighted equally. Change a status from the dropdown and every score, including the Summary, recalculates.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>STAKEHOLDER ALIGNMENT</t>
         </is>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="33">
         <f>(COUNTIF(A8:A13,"Yes")+0.5*COUNTIF(A8:A13,"In Progress"))/COUNTA($B$8:$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="A8" s="34" t="n"/>
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Champion identified and confirmed (has influence + is actively selling internally)</t>
         </is>
@@ -1404,8 +1432,8 @@
       <c r="C8" s="12" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="34" t="inlineStr">
+      <c r="A9" s="34" t="n"/>
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>Economic buyer identified and engaged directly (not just through champion)</t>
         </is>
@@ -1413,8 +1441,8 @@
       <c r="C9" s="12" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="33" t="n"/>
-      <c r="B10" s="34" t="inlineStr">
+      <c r="A10" s="34" t="n"/>
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>All stakeholders/influencers mapped (security, legal, procurement, end users, IT)</t>
         </is>
@@ -1422,8 +1450,8 @@
       <c r="C10" s="12" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="34" t="inlineStr">
+      <c r="A11" s="34" t="n"/>
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Decision criteria documented and agreed by buyer</t>
         </is>
@@ -1431,8 +1459,8 @@
       <c r="C11" s="12" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="33" t="n"/>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="A12" s="34" t="n"/>
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Decision process and approval chain confirmed (who signs, in what order)</t>
         </is>
@@ -1440,8 +1468,8 @@
       <c r="C12" s="12" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="A13" s="34" t="n"/>
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>Compelling event / reason to act by target date is explicit</t>
         </is>
@@ -1449,19 +1477,19 @@
       <c r="C13" s="12" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>TECHNICAL VALIDATION</t>
         </is>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="33">
         <f>(COUNTIF(A16:A19,"Yes")+0.5*COUNTIF(A16:A19,"In Progress"))/COUNTA($B$16:$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="33" t="n"/>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="A16" s="34" t="n"/>
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>Technical win confirmed (POC/trial success criteria met and documented)</t>
         </is>
@@ -1469,8 +1497,8 @@
       <c r="C16" s="12" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="33" t="n"/>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="A17" s="34" t="n"/>
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Security review status known (in progress / passed / not started)</t>
         </is>
@@ -1478,8 +1506,8 @@
       <c r="C17" s="12" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="33" t="n"/>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="A18" s="34" t="n"/>
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>Integration requirements scoped and no blockers open</t>
         </is>
@@ -1487,8 +1515,8 @@
       <c r="C18" s="12" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="33" t="n"/>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="A19" s="34" t="n"/>
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>Any outstanding product gaps or feature requests flagged to product team</t>
         </is>
@@ -1496,19 +1524,19 @@
       <c r="C19" s="12" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>COMMERCIAL</t>
         </is>
       </c>
-      <c r="C21" s="32">
+      <c r="C21" s="33">
         <f>(COUNTIF(A22:A27,"Yes")+0.5*COUNTIF(A22:A27,"In Progress"))/COUNTA($B$22:$B$27)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="33" t="n"/>
-      <c r="B22" s="34" t="inlineStr">
+      <c r="A22" s="34" t="n"/>
+      <c r="B22" s="35" t="inlineStr">
         <is>
           <t>Budget confirmed to exist and be allocated for this fiscal period</t>
         </is>
@@ -1516,8 +1544,8 @@
       <c r="C22" s="12" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="33" t="n"/>
-      <c r="B23" s="34" t="inlineStr">
+      <c r="A23" s="34" t="n"/>
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Pricing/packaging aligned with buyer's expectations</t>
         </is>
@@ -1525,8 +1553,8 @@
       <c r="C23" s="12" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="33" t="n"/>
-      <c r="B24" s="34" t="inlineStr">
+      <c r="A24" s="34" t="n"/>
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Quote/order form sent and reviewed by buyer</t>
         </is>
@@ -1534,8 +1562,8 @@
       <c r="C24" s="12" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="33" t="n"/>
-      <c r="B25" s="34" t="inlineStr">
+      <c r="A25" s="34" t="n"/>
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>Procurement process started (vendor onboarding, security questionnaires, etc.)</t>
         </is>
@@ -1543,8 +1571,8 @@
       <c r="C25" s="12" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="33" t="n"/>
-      <c r="B26" s="34" t="inlineStr">
+      <c r="A26" s="34" t="n"/>
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>Legal/MSA redlines identified early, not first surfaced at the finish line</t>
         </is>
@@ -1552,8 +1580,8 @@
       <c r="C26" s="12" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="33" t="n"/>
-      <c r="B27" s="34" t="inlineStr">
+      <c r="A27" s="34" t="n"/>
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>Have we established enough value w/ key stakeholders to mitigate potential for discounting?</t>
         </is>
@@ -1561,19 +1589,19 @@
       <c r="C27" s="12" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>COMPETITION</t>
         </is>
       </c>
-      <c r="C29" s="32">
+      <c r="C29" s="33">
         <f>(COUNTIF(A30:A32,"Yes")+0.5*COUNTIF(A30:A32,"In Progress"))/COUNTA($B$30:$B$32)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="33" t="n"/>
-      <c r="B30" s="34" t="inlineStr">
+      <c r="A30" s="34" t="n"/>
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>Competitive landscape known (incumbent, alternatives being evaluated)</t>
         </is>
@@ -1581,8 +1609,8 @@
       <c r="C30" s="12" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="33" t="n"/>
-      <c r="B31" s="34" t="inlineStr">
+      <c r="A31" s="34" t="n"/>
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>Differentiation validated with champion, they can repeat it internally</t>
         </is>
@@ -1590,8 +1618,8 @@
       <c r="C31" s="12" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="33" t="n"/>
-      <c r="B32" s="34" t="inlineStr">
+      <c r="A32" s="34" t="n"/>
+      <c r="B32" s="35" t="inlineStr">
         <is>
           <t>No unaddressed objections tied to a competitor's pitch</t>
         </is>
@@ -1599,19 +1627,19 @@
       <c r="C32" s="12" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="32" t="inlineStr">
         <is>
           <t>TIMELINE &amp; RISK</t>
         </is>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="33">
         <f>(COUNTIF(A35:A41,"Yes")+0.5*COUNTIF(A35:A41,"In Progress"))/COUNTA($B$35:$B$41)</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="33" t="n"/>
-      <c r="B35" s="34" t="inlineStr">
+      <c r="A35" s="34" t="n"/>
+      <c r="B35" s="35" t="inlineStr">
         <is>
           <t>Mutual close plan shared with buyer, with dates both sides agreed to</t>
         </is>
@@ -1619,8 +1647,8 @@
       <c r="C35" s="12" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="33" t="n"/>
-      <c r="B36" s="34" t="inlineStr">
+      <c r="A36" s="34" t="n"/>
+      <c r="B36" s="35" t="inlineStr">
         <is>
           <t>Next step scheduled with a specific date (not "follow up next week")</t>
         </is>
@@ -1628,8 +1656,8 @@
       <c r="C36" s="12" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="33" t="n"/>
-      <c r="B37" s="34" t="inlineStr">
+      <c r="A37" s="34" t="n"/>
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>Key risk(s) to close named explicitly, e.g. budget freeze, exec turnover, competing priority</t>
         </is>
@@ -1637,8 +1665,8 @@
       <c r="C37" s="12" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="33" t="n"/>
-      <c r="B38" s="34" t="inlineStr">
+      <c r="A38" s="34" t="n"/>
+      <c r="B38" s="35" t="inlineStr">
         <is>
           <t>Backup plan if primary champion goes dark or leaves</t>
         </is>
@@ -1646,8 +1674,8 @@
       <c r="C38" s="12" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="33" t="n"/>
-      <c r="B39" s="34" t="inlineStr">
+      <c r="A39" s="34" t="n"/>
+      <c r="B39" s="35" t="inlineStr">
         <is>
           <t>Do we have a clear migration or onboarding plan?</t>
         </is>
@@ -1655,8 +1683,8 @@
       <c r="C39" s="12" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="33" t="n"/>
-      <c r="B40" s="34" t="inlineStr">
+      <c r="A40" s="34" t="n"/>
+      <c r="B40" s="35" t="inlineStr">
         <is>
           <t>Do we have an onboarding owner identified?</t>
         </is>
@@ -1664,8 +1692,8 @@
       <c r="C40" s="12" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="33" t="n"/>
-      <c r="B41" s="34" t="inlineStr">
+      <c r="A41" s="34" t="n"/>
+      <c r="B41" s="35" t="inlineStr">
         <is>
           <t>Forecast category matches actual deal signals (don't call it Commit if 3+ boxes above are unchecked)</t>
         </is>
@@ -1673,14 +1701,14 @@
       <c r="C41" s="12" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="35" t="inlineStr">
+      <c r="A43" s="36" t="inlineStr">
         <is>
           <t>COVERAGE AND EVIDENCE LIMITS</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14.5" customHeight="1">
-      <c r="A44" s="36" t="n"/>
+      <c r="A44" s="37" t="n"/>
     </row>
     <row r="45" ht="14.5" customHeight="1"/>
     <row r="46" ht="14.5" customHeight="1"/>
@@ -1724,46 +1752,46 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Action Plan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="37" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>One row per Health Score item that is not a Yes. Filter by owner or status.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="31" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="B3" s="31" t="inlineStr">
+      <c r="B3" s="32" t="inlineStr">
         <is>
           <t>Gap (from Health Score)</t>
         </is>
       </c>
-      <c r="C3" s="31" t="inlineStr">
+      <c r="C3" s="32" t="inlineStr">
         <is>
           <t>Recommended Action</t>
         </is>
       </c>
-      <c r="D3" s="31" t="inlineStr">
+      <c r="D3" s="32" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E3" s="31" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="31" t="inlineStr">
+      <c r="F3" s="32" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
@@ -1799,14 +1827,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Stakeholder Map</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>BUYING COMMITTEE: seniority x function</t>
         </is>
@@ -1819,132 +1847,132 @@
       <c r="G3" s="12" t="n"/>
     </row>
     <row r="5" ht="31.5" customHeight="1">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>C-Suite</t>
         </is>
       </c>
-      <c r="B5" s="40" t="n"/>
+      <c r="B5" s="41" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Seniority</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Business / LOB</t>
         </is>
       </c>
-      <c r="C7" s="41" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Technical / Engineering</t>
         </is>
       </c>
-      <c r="D7" s="41" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Enablement / Ops</t>
         </is>
       </c>
-      <c r="E7" s="41" t="inlineStr">
+      <c r="E7" s="42" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="F7" s="41" t="inlineStr">
+      <c r="F7" s="42" t="inlineStr">
         <is>
           <t>IT / Platform</t>
         </is>
       </c>
-      <c r="G7" s="41" t="inlineStr">
+      <c r="G7" s="42" t="inlineStr">
         <is>
           <t>Procurement / Legal</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>VP</t>
         </is>
       </c>
-      <c r="B8" s="43" t="n"/>
-      <c r="C8" s="43" t="n"/>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="43" t="n"/>
-      <c r="F8" s="43" t="n"/>
-      <c r="G8" s="43" t="n"/>
+      <c r="B8" s="44" t="n"/>
+      <c r="C8" s="44" t="n"/>
+      <c r="D8" s="44" t="n"/>
+      <c r="E8" s="44" t="n"/>
+      <c r="F8" s="44" t="n"/>
+      <c r="G8" s="44" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="A9" s="43" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="B9" s="43" t="n"/>
-      <c r="C9" s="43" t="n"/>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="43" t="n"/>
-      <c r="F9" s="43" t="n"/>
-      <c r="G9" s="43" t="n"/>
+      <c r="B9" s="44" t="n"/>
+      <c r="C9" s="44" t="n"/>
+      <c r="D9" s="44" t="n"/>
+      <c r="E9" s="44" t="n"/>
+      <c r="F9" s="44" t="n"/>
+      <c r="G9" s="44" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="B10" s="43" t="n"/>
-      <c r="C10" s="43" t="n"/>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="43" t="n"/>
-      <c r="F10" s="43" t="n"/>
-      <c r="G10" s="43" t="n"/>
+      <c r="B10" s="44" t="n"/>
+      <c r="C10" s="44" t="n"/>
+      <c r="D10" s="44" t="n"/>
+      <c r="E10" s="44" t="n"/>
+      <c r="F10" s="44" t="n"/>
+      <c r="G10" s="44" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="42" t="inlineStr">
+      <c r="A11" s="43" t="inlineStr">
         <is>
           <t>Individual Contributor</t>
         </is>
       </c>
-      <c r="B11" s="43" t="n"/>
-      <c r="C11" s="43" t="n"/>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="43" t="n"/>
-      <c r="F11" s="43" t="n"/>
-      <c r="G11" s="43" t="n"/>
+      <c r="B11" s="44" t="n"/>
+      <c r="C11" s="44" t="n"/>
+      <c r="D11" s="44" t="n"/>
+      <c r="E11" s="44" t="n"/>
+      <c r="F11" s="44" t="n"/>
+      <c r="G11" s="44" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="42" t="inlineStr">
+      <c r="A12" s="43" t="inlineStr">
         <is>
           <t>Seniority not stated</t>
         </is>
       </c>
-      <c r="B12" s="43" t="n"/>
-      <c r="C12" s="43" t="n"/>
-      <c r="D12" s="43" t="n"/>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
+      <c r="B12" s="44" t="n"/>
+      <c r="C12" s="44" t="n"/>
+      <c r="D12" s="44" t="n"/>
+      <c r="E12" s="44" t="n"/>
+      <c r="F12" s="44" t="n"/>
+      <c r="G12" s="44" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="44" t="inlineStr">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B14" s="45" t="inlineStr">
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Engaged</t>
         </is>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>Emerging / not direct</t>
         </is>
       </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="D14" s="48" t="inlineStr">
         <is>
           <t>Not yet mapped</t>
         </is>
@@ -1952,114 +1980,114 @@
     </row>
     <row r="15" ht="25.5" customHeight="1"/>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="48" t="inlineStr">
+      <c r="A16" s="49" t="inlineStr">
         <is>
           <t>KEY PERSONAS</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr">
         <is>
           <t>Engagement</t>
         </is>
       </c>
-      <c r="D17" s="31" t="inlineStr">
+      <c r="D17" s="32" t="inlineStr">
         <is>
           <t>Notes / Gap</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="49" t="inlineStr">
+      <c r="A18" s="50" t="inlineStr">
         <is>
           <t>Economic Buyer</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="33" t="n"/>
-      <c r="D18" s="20" t="n"/>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="21" t="n"/>
       <c r="E18" s="12" t="n"/>
       <c r="F18" s="12" t="n"/>
       <c r="G18" s="12" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="49" t="inlineStr">
+      <c r="A19" s="50" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
       </c>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="33" t="n"/>
-      <c r="D19" s="20" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="34" t="n"/>
+      <c r="D19" s="21" t="n"/>
       <c r="E19" s="12" t="n"/>
       <c r="F19" s="12" t="n"/>
       <c r="G19" s="12" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="49" t="inlineStr">
+      <c r="A20" s="50" t="inlineStr">
         <is>
           <t>Executive Sponsor</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="33" t="n"/>
-      <c r="D20" s="20" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="34" t="n"/>
+      <c r="D20" s="21" t="n"/>
       <c r="E20" s="12" t="n"/>
       <c r="F20" s="12" t="n"/>
       <c r="G20" s="12" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
+      <c r="A21" s="50" t="inlineStr">
         <is>
           <t>Influencer 1 - Security / Legal</t>
         </is>
       </c>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="33" t="n"/>
-      <c r="D21" s="20" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="21" t="n"/>
       <c r="E21" s="12" t="n"/>
       <c r="F21" s="12" t="n"/>
       <c r="G21" s="12" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="49" t="inlineStr">
+      <c r="A22" s="50" t="inlineStr">
         <is>
           <t>Influencer 2 - Procurement</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="20" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="21" t="n"/>
       <c r="E22" s="12" t="n"/>
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="12" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
+      <c r="A23" s="50" t="inlineStr">
         <is>
           <t>Influencer 3 - End Users / IT</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="33" t="n"/>
-      <c r="D23" s="20" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="34" t="n"/>
+      <c r="D23" s="21" t="n"/>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="12" t="n"/>
       <c r="G23" s="12" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="50" t="inlineStr">
+      <c r="A25" s="51" t="inlineStr">
         <is>
           <t>Open question: Do we have a text relationship with any of these contacts?</t>
         </is>

</xml_diff>